<commit_message>
Atualização do banco, processador e tratamento para deixar de forma correta com o padrão exigido
</commit_message>
<xml_diff>
--- a/resultados/relatorio_final.xlsx
+++ b/resultados/relatorio_final.xlsx
@@ -151,8 +151,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Legenda_Fase_5" displayName="Legenda_Fase_5" ref="A19:D29" headerRowCount="1">
-  <autoFilter ref="A19:D29"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Legenda_Fase_5" displayName="Legenda_Fase_5" ref="A19:D28" headerRowCount="1">
+  <autoFilter ref="A19:D28"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Cód. (Turma)"/>
     <tableColumn id="2" name="Nome da Disciplina"/>
@@ -179,8 +179,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Legenda_Fase_6" displayName="Legenda_Fase_6" ref="A19:D26" headerRowCount="1">
-  <autoFilter ref="A19:D26"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Legenda_Fase_6" displayName="Legenda_Fase_6" ref="A19:D27" headerRowCount="1">
+  <autoFilter ref="A19:D27"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Cód. (Turma)"/>
     <tableColumn id="2" name="Nome da Disciplina"/>
@@ -248,8 +248,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Legenda_Fase_3" displayName="Legenda_Fase_3" ref="A19:D35" headerRowCount="1">
-  <autoFilter ref="A19:D35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Legenda_Fase_3" displayName="Legenda_Fase_3" ref="A19:D34" headerRowCount="1">
+  <autoFilter ref="A19:D34"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Cód. (Turma)"/>
     <tableColumn id="2" name="Nome da Disciplina"/>
@@ -276,8 +276,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Legenda_Fase_4" displayName="Legenda_Fase_4" ref="A19:D30" headerRowCount="1">
-  <autoFilter ref="A19:D30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Legenda_Fase_4" displayName="Legenda_Fase_4" ref="A19:D34" headerRowCount="1">
+  <autoFilter ref="A19:D34"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Cód. (Turma)"/>
     <tableColumn id="2" name="Nome da Disciplina"/>
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>3ª Fase</t>
+          <t>2ª Fase</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2ª Fase</t>
+          <t>4ª Fase</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3284,12 +3284,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>5ª Fase (Optativa)</t>
+          <t>4ª Fase</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>Obrigatória</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>5ª Fase (Optativa)</t>
+          <t>5ª Fase</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>6ª Fase (Optativa)</t>
+          <t>6ª Fase</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>5ª Fase (Optativa)</t>
+          <t>5ª Fase</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>6ª Fase</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>6ª Fase (Optativa)</t>
+          <t>5ª Fase</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>5ª Fase (Optativa)</t>
+          <t>6ª Fase</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>5ª Fase (Optativa)</t>
+          <t>5ª Fase</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>6ª Fase (Optativa)</t>
+          <t>6ª Fase</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4560,6 +4560,130 @@
       <c r="L64" t="inlineStr">
         <is>
           <t>Francisco Carlos Caramello Junior</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026.2</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>INE5111</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>02342A</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Estatística Aplicada I</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>4ª Fase</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Obrigatória</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>3.0820-2 | 4.1010-2</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>CED-LBPREV | CED-LBPREV</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Vera do Carmo Comparsi de Vargas</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026.2</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>INE5111</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>02342C</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Estatística Aplicada I</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>4ª Fase</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Obrigatória</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>2.1830-2 | 5.1830-2</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>CED-LBPREV | CED-102 C</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Manoella Reis Cardenuto</t>
         </is>
       </c>
     </row>
@@ -5505,7 +5629,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CIN7412 (04342A)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -5537,7 +5661,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CIN7412 (04342A)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -5734,7 +5858,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7309 (02342C)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5766,7 +5890,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7309 (02342C)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5798,7 +5922,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7309 (02342C)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5830,7 +5954,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7309 (02342C)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5922,29 +6046,29 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CIN7412 (02342C)</t>
+          <t>CIN7309 (02342C)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Marketing da Informação</t>
+          <t>Gestão de Processos Organizacionais</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AUX-ALOCAR</t>
+          <t>CED-LBTEC</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sabrina Borges Ramos de Carvalho</t>
+          <t>?</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CIN7412 (04342A)</t>
+          <t>CIN7412 (02342C)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5954,12 +6078,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CED-004 D</t>
+          <t>AUX-ALOCAR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sonali Paula Molin Bedin</t>
+          <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
       </c>
     </row>
@@ -6044,7 +6168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6425,7 +6549,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CIN7309 (02342C)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6457,7 +6581,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CIN7309 (02342C)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6489,7 +6613,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CIN7309 (02342C)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6521,7 +6645,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CIN7309 (02342C)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6789,7 +6913,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CIN7309 (02342C)</t>
+          <t>CIN7309 (03342A)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6811,29 +6935,29 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CIN7309 (03342A)</t>
+          <t>CIN7936 (03342A)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Gestão de Processos Organizacionais</t>
+          <t>Proteção de Dados Pessoais</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CED-LBTEC</t>
+          <t>CED-LBPREV</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Marcelo Minghelli</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CIN7936 (03342A)</t>
+          <t>CIN7936 (03342C)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6843,7 +6967,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CED-LBPREV</t>
+          <t>CED-102 C</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -6855,29 +6979,29 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CIN7936 (03342C)</t>
+          <t>HST7921 (03342A)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Proteção de Dados Pessoais</t>
+          <t>História do Brasil Contemporâneo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CED-102 C</t>
+          <t>CED-LBPREV</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Marcelo Minghelli</t>
+          <t>Roselane Neckel</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>HST7921 (03342A)</t>
+          <t>HST7921 (03342C)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6891,28 +7015,6 @@
         </is>
       </c>
       <c r="D34" t="inlineStr">
-        <is>
-          <t>Roselane Neckel</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>HST7921 (03342C)</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>História do Brasil Contemporâneo</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>CED-LBPREV</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
         <is>
           <t>Roselane Neckel</t>
         </is>
@@ -6933,12 +7035,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
@@ -7021,7 +7123,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>INE5111 (02342A)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -7053,7 +7155,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>INE5111 (02342A)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -7085,12 +7187,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7412 (04342A)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>INE5111 (02342A)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7117,12 +7219,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7412 (04342A)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>INE5111 (02342A)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -7304,12 +7406,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>INE5111 (02342C)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CIN7401 (04342C)</t>
+          <t>CIN7401 (04342C) / CIN7903 (06342)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -7319,7 +7421,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>INE5111 (02342C)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -7336,12 +7438,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>INE5111 (02342C)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CIN7401 (04342C)</t>
+          <t>CIN7401 (04342C) / CIN7903 (06342)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -7351,7 +7453,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>INE5111 (02342C)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -7694,6 +7796,94 @@
       <c r="D30" t="inlineStr">
         <is>
           <t>Sabrina Borges Ramos de Carvalho</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CIN7412 (04342A)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Marketing da Informação</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CED-004 D</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Sonali Paula Molin Bedin</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CIN7903 (06342)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Inteligência Competitiva</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>AUX-ALOCAR</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>INE5111 (02342A)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Estatística Aplicada I</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CED-LBPREV | CED-LBPREV</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Vera do Carmo Comparsi de Vargas</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>INE5111 (02342C)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Estatística Aplicada I</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CED-LBPREV | CED-102 C</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Manoella Reis Cardenuto</t>
         </is>
       </c>
     </row>
@@ -7712,14 +7902,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -8088,7 +8278,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CIN7903 (06342)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -8098,7 +8288,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CIN7904 (06342)</t>
+          <t>CIN7904 (06342) / CIN7935 (06342)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -8120,7 +8310,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CIN7903 (06342)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -8130,7 +8320,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CIN7904 (06342)</t>
+          <t>CIN7904 (06342) / CIN7935 (06342)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -8152,7 +8342,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CIN7938 (05342)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -8184,7 +8374,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CIN7938 (05342)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -8347,12 +8537,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CIN7903 (06342)</t>
+          <t>CIN7904 (06342)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Inteligência Competitiva</t>
+          <t>Avaliação de Desempenho</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -8362,19 +8552,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CIN7904 (06342)</t>
+          <t>CIN7917 (05342)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Avaliação de Desempenho</t>
+          <t>Visualização da Informação</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -8384,41 +8574,41 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sabrina Borges Ramos de Carvalho</t>
+          <t>Márcio Matias</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CIN7917 (05342)</t>
+          <t>CIN7935 (06342)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Visualização da Informação</t>
+          <t>Liderança e Gerência</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AUX-ALOCAR</t>
+          <t>CED-LBCON</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Márcio Matias</t>
+          <t>Sonali Paula Molin Bedin</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CIN7938 (05342)</t>
+          <t>CIN7945 (05342)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Segurança da Informação</t>
+          <t>Fontes de Informação Tecnológica</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -8427,28 +8617,6 @@
         </is>
       </c>
       <c r="D28" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>CIN7945 (05342)</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Fontes de Informação Tecnológica</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>AUX-ALOCAR</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
         <is>
           <t>Márcio Matias</t>
         </is>
@@ -8469,11 +8637,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -8840,7 +9008,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CIN7603 (06342)</t>
+          <t>CIN7603 (06342) / CIN7927 (05342)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -8855,7 +9023,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CIN7935 (06342)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -8872,7 +9040,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CIN7603 (06342)</t>
+          <t>CIN7603 (06342) / CIN7927 (05342)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -8887,7 +9055,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CIN7935 (06342)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -8909,7 +9077,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7938 (05342)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -8941,7 +9109,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7938 (05342)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -9104,42 +9272,64 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CIN7935 (06342)</t>
+          <t>CIN7927 (05342)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Liderança e Gerência</t>
+          <t>Gestão da Informação Pública</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CED-LBCON</t>
+          <t>AUX-ALOCAR</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Sonali Paula Molin Bedin</t>
+          <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>CIN7938 (05342)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>AUX-ALOCAR</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>CIN7946 (05342)</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Pitch de Carreira</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>CED-LBCON</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Sonali Paula Molin Bedin</t>
         </is>

</xml_diff>